<commit_message>
Regenerate sample report with the final code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ax3VGeapDUVfTHWoVdgXik
</commit_message>
<xml_diff>
--- a/data/sample/sample_report.xlsx
+++ b/data/sample/sample_report.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ERP_vs_CAD'!$A$1:$K$55</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'ERP_vs_CAD'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Errors_Skipped'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Metrics'!$A$3:$K$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Metrics'!$A$3:$L$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -858,7 +858,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-01 14:23</t>
+          <t>2026-10-01 14:45</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
     </row>
     <row r="42">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -970,167 +970,167 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>time: geometry_per_file_max_s</t>
+          <t>time: geometry_s</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>2.94</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>time: geometry_per_file_mean_s</t>
+          <t>time: geometry_unique</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>0.26</v>
+        <v>54</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>time: geometry_per_file_median_s</t>
+          <t>time: geometry_wall_s</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>time: geometry_per_file_p90_s</t>
+          <t>time: scan_s</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>0.57</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>time: geometry_s</t>
+          <t>time: scoring_s</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>7</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>time: geometry_unique</t>
+          <t>time: shape_checks</t>
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>time: geometry_wall_s</t>
+          <t>time: shape_s</t>
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>7</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>time: scan_s</t>
+          <t>time: total_s</t>
         </is>
       </c>
       <c r="B51" s="7" t="n">
-        <v>0.92</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>time: scoring_s</t>
+          <t>threshold: geo_exact</t>
         </is>
       </c>
       <c r="B52" s="7" t="n">
-        <v>2.08</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>time: shape_checks</t>
+          <t>threshold: geo_identical</t>
         </is>
       </c>
       <c r="B53" s="7" t="n">
-        <v>22</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>time: shape_s</t>
+          <t>threshold: geo_near</t>
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>2.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>time: total_s</t>
+          <t>threshold: geo_split_type_tol</t>
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>10.38</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>threshold: geo_exact</t>
+          <t>threshold: near_max_face_ratio</t>
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>1e-06</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>threshold: geo_identical</t>
+          <t>threshold: near_max_type_dist</t>
         </is>
       </c>
       <c r="B57" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>threshold: geo_near</t>
+          <t>threshold: unit_tol</t>
         </is>
       </c>
       <c r="B58" s="7" t="n">
-        <v>0.1</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>threshold: geo_split_type_tol</t>
+          <t>threshold: name_similar</t>
         </is>
       </c>
       <c r="B59" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>threshold: near_max_face_ratio</t>
+          <t>threshold: name_k0</t>
         </is>
       </c>
       <c r="B60" s="7" t="n">
@@ -1140,37 +1140,37 @@
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>threshold: near_max_type_dist</t>
+          <t>threshold: name_partial_factor</t>
         </is>
       </c>
       <c r="B61" s="7" t="n">
-        <v>0.25</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>threshold: unit_tol</t>
+          <t>threshold: name_candidate</t>
         </is>
       </c>
       <c r="B62" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>threshold: name_similar</t>
+          <t>threshold: shape_same_excess50</t>
         </is>
       </c>
       <c r="B63" s="7" t="n">
-        <v>0.9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>threshold: name_k0</t>
+          <t>threshold: shape_near_excess50</t>
         </is>
       </c>
       <c r="B64" s="7" t="n">
@@ -1180,70 +1180,30 @@
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>threshold: name_partial_factor</t>
+          <t>threshold: shape_near_p95</t>
         </is>
       </c>
       <c r="B65" s="7" t="n">
-        <v>0.85</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>threshold: name_candidate</t>
+          <t>threshold: mirror_ratio</t>
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>threshold: shape_same_excess50</t>
+          <t>threshold: skew_min</t>
         </is>
       </c>
       <c r="B67" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>threshold: shape_near_excess50</t>
-        </is>
-      </c>
-      <c r="B68" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="7" t="inlineStr">
-        <is>
-          <t>threshold: shape_near_p95</t>
-        </is>
-      </c>
-      <c r="B69" s="7" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>threshold: mirror_ratio</t>
-        </is>
-      </c>
-      <c r="B70" s="7" t="n">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>threshold: skew_min</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="n">
         <v>0.004</v>
       </c>
     </row>
@@ -8441,20 +8401,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="70" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8472,50 +8433,55 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>GT pairs</t>
+          <t>GT pairs (recall)</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>Found</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>Missed</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>FP</t>
+          <t>Predicted (precision)</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
+          <t>Wrong</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
           <t>Precision</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>Recall</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>Met?</t>
         </is>
       </c>
-      <c r="K3" s="8" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>How it is counted</t>
         </is>
@@ -8537,10 +8503,10 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="n">
         <v>0</v>
-      </c>
-      <c r="F4" s="16" t="n">
-        <v>1</v>
       </c>
       <c r="G4" s="16" t="n">
         <v>1</v>
@@ -8548,17 +8514,20 @@
       <c r="H4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>P&gt;=95% and R&gt;=95%</t>
         </is>
       </c>
-      <c r="J4" s="17" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>(base, A) pairs proposed as merge candidates; precision over merge candidates with a A file</t>
         </is>
@@ -8580,10 +8549,10 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="n">
         <v>0</v>
-      </c>
-      <c r="F5" s="16" t="n">
-        <v>1</v>
       </c>
       <c r="G5" s="16" t="n">
         <v>1</v>
@@ -8591,17 +8560,20 @@
       <c r="H5" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>P&gt;=95% and R&gt;=95%</t>
         </is>
       </c>
-      <c r="J5" s="17" t="inlineStr">
+      <c r="K5" s="17" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>(base, B) pairs proposed as merge candidates; precision over merge candidates with a B file</t>
         </is>
@@ -8623,10 +8595,10 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="n">
         <v>0</v>
-      </c>
-      <c r="F6" s="16" t="n">
-        <v>1</v>
       </c>
       <c r="G6" s="16" t="n">
         <v>1</v>
@@ -8634,17 +8606,20 @@
       <c r="H6" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>P&gt;=95% and R&gt;=95%</t>
         </is>
       </c>
-      <c r="J6" s="17" t="inlineStr">
+      <c r="K6" s="17" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>(base, C) pairs proposed as merge candidates; precision over merge candidates with a C file</t>
         </is>
@@ -8666,10 +8641,10 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="n">
         <v>0</v>
-      </c>
-      <c r="F7" s="16" t="n">
-        <v>1</v>
       </c>
       <c r="G7" s="16" t="n">
         <v>1</v>
@@ -8677,17 +8652,20 @@
       <c r="H7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>P&gt;=95% and R&gt;=95%</t>
         </is>
       </c>
-      <c r="J7" s="17" t="inlineStr">
+      <c r="K7" s="17" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>(base, D) pairs proposed as merge candidates; precision over merge candidates with a D file</t>
         </is>
@@ -8709,10 +8687,10 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" t="n">
         <v>0</v>
-      </c>
-      <c r="F8" s="16" t="n">
-        <v>1</v>
       </c>
       <c r="G8" s="16" t="n">
         <v>1</v>
@@ -8720,17 +8698,20 @@
       <c r="H8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>R&gt;=80% at P&gt;=90%</t>
         </is>
       </c>
-      <c r="J8" s="17" t="inlineStr">
+      <c r="K8" s="17" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>(base, E) pairs predicted near-identical; precision over near predictions with an E file</t>
         </is>
@@ -8752,28 +8733,31 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="G9" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="H9" s="16" t="n">
         <v>0.75</v>
       </c>
-      <c r="H9" s="16" t="n">
+      <c r="I9" t="n">
         <v>0.7742</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>F1&gt;=0.85</t>
         </is>
       </c>
-      <c r="J9" s="12" t="inlineStr">
+      <c r="K9" s="12" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>name layer only: (base, F) pairs with name score &gt;= threshold; precision over links with an F file (same GT group = correct)</t>
         </is>
@@ -8794,22 +8778,21 @@
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="16" t="n"/>
-      <c r="G10" s="16" t="n">
+      <c r="G10" s="16" t="n"/>
+      <c r="H10" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="16" t="n"/>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>(base, F) pairs predicted identical by L1/L3 (F files are copies/re-exports)</t>
         </is>
@@ -8824,25 +8807,24 @@
       <c r="C11" t="n">
         <v>17</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="G11" s="16" t="n">
         <v>0.8947000000000001</v>
       </c>
-      <c r="G11" s="16" t="n"/>
       <c r="H11" s="16" t="n"/>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>all pairs with name score &gt;= threshold; precision = share within the same GT group</t>
         </is>
@@ -8860,23 +8842,22 @@
       <c r="C12" t="n">
         <v>25</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="16" t="n"/>
       <c r="G12" s="16" t="n"/>
       <c r="H12" s="16" t="n"/>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>FP &lt;= 2%</t>
         </is>
       </c>
-      <c r="J12" s="17" t="inlineStr">
+      <c r="K12" s="17" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>FP rate = 0.0: flagged = merge candidates + near-identical alerts; FP = different GT groups</t>
         </is>
@@ -8897,22 +8878,21 @@
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="16" t="n"/>
-      <c r="G13" s="16" t="n">
+      <c r="G13" s="16" t="n"/>
+      <c r="H13" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="16" t="n"/>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>share handled correctly; category=identical_attr_conflict: 3</t>
         </is>
@@ -8933,22 +8913,21 @@
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="16" t="n"/>
-      <c r="G14" s="16" t="n">
+      <c r="G14" s="16" t="n"/>
+      <c r="H14" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="16" t="n"/>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>share handled correctly; category=mirror: 1</t>
         </is>
@@ -8969,22 +8948,21 @@
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="16" t="n"/>
-      <c r="G15" s="16" t="n">
+      <c r="G15" s="16" t="n"/>
+      <c r="H15" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="16" t="n"/>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>share handled correctly; category=none: 3</t>
         </is>
@@ -9005,22 +8983,21 @@
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="16" t="n"/>
-      <c r="G16" s="16" t="n">
+      <c r="G16" s="16" t="n"/>
+      <c r="H16" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="16" t="n"/>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>share handled correctly; category=name_similar: 1, category=none: 2</t>
         </is>
@@ -9087,7 +9064,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K16"/>
+  <autoFilter ref="A3:L16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>